<commit_message>
inner merge target and features
</commit_message>
<xml_diff>
--- a/data/ABS_census_features.xlsx
+++ b/data/ABS_census_features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2d59a5571354f26b/Documents/2026 - semester 2/Case Studies for Data Science/Individual A1/Ind A1 Repo/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{2F8066A8-613E-44DA-854D-36CAB6FE5108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{737892B3-767C-470A-8B70-66DB3E26A978}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{2F8066A8-613E-44DA-854D-36CAB6FE5108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18CAE7CA-04EB-4A17-BC40-601219805DBD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4AC0AC66-49F0-4C0B-B9FC-0FF9AEA9BF84}"/>
   </bookViews>
@@ -110,9 +110,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>SA2_CODE_2021</t>
-  </si>
-  <si>
     <t>Median_tot_prsnl_inc_weekly</t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>Tot_Indigenous_%</t>
+  </si>
+  <si>
+    <t>Code</t>
   </si>
 </sst>
 </file>
@@ -592,40 +592,40 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
@@ -3550,8 +3550,8 @@
       <c r="K78">
         <v>0</v>
       </c>
-      <c r="L78" t="e">
-        <v>#DIV/0!</v>
+      <c r="L78">
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.35">
@@ -14836,8 +14836,8 @@
       <c r="K375">
         <v>0</v>
       </c>
-      <c r="L375" t="e">
-        <v>#DIV/0!</v>
+      <c r="L375">
+        <v>0</v>
       </c>
     </row>
     <row r="376" spans="1:12" x14ac:dyDescent="0.35">
@@ -25058,8 +25058,8 @@
       <c r="K644">
         <v>0</v>
       </c>
-      <c r="L644" t="e">
-        <v>#DIV/0!</v>
+      <c r="L644">
+        <v>0</v>
       </c>
     </row>
     <row r="645" spans="1:12" x14ac:dyDescent="0.35">
@@ -28364,8 +28364,8 @@
       <c r="K731">
         <v>0</v>
       </c>
-      <c r="L731" t="e">
-        <v>#DIV/0!</v>
+      <c r="L731">
+        <v>0</v>
       </c>
     </row>
     <row r="732" spans="1:12" x14ac:dyDescent="0.35">
@@ -28478,8 +28478,8 @@
       <c r="K734">
         <v>0</v>
       </c>
-      <c r="L734" t="e">
-        <v>#DIV/0!</v>
+      <c r="L734">
+        <v>0</v>
       </c>
     </row>
     <row r="735" spans="1:12" x14ac:dyDescent="0.35">
@@ -30226,8 +30226,8 @@
       <c r="K780">
         <v>0</v>
       </c>
-      <c r="L780" t="e">
-        <v>#DIV/0!</v>
+      <c r="L780">
+        <v>0</v>
       </c>
     </row>
     <row r="781" spans="1:12" x14ac:dyDescent="0.35">
@@ -30416,8 +30416,8 @@
       <c r="K785">
         <v>0</v>
       </c>
-      <c r="L785" t="e">
-        <v>#DIV/0!</v>
+      <c r="L785">
+        <v>0</v>
       </c>
     </row>
     <row r="786" spans="1:12" x14ac:dyDescent="0.35">
@@ -48922,8 +48922,8 @@
       <c r="K1272">
         <v>0</v>
       </c>
-      <c r="L1272" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1272">
+        <v>0</v>
       </c>
     </row>
     <row r="1273" spans="1:12" x14ac:dyDescent="0.35">
@@ -53444,8 +53444,8 @@
       <c r="K1391">
         <v>0</v>
       </c>
-      <c r="L1391" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1391">
+        <v>0</v>
       </c>
     </row>
     <row r="1392" spans="1:12" x14ac:dyDescent="0.35">
@@ -55952,8 +55952,8 @@
       <c r="K1457">
         <v>0</v>
       </c>
-      <c r="L1457" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1457">
+        <v>0</v>
       </c>
     </row>
     <row r="1458" spans="1:12" x14ac:dyDescent="0.35">
@@ -57358,8 +57358,8 @@
       <c r="K1494">
         <v>0</v>
       </c>
-      <c r="L1494" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1494">
+        <v>0</v>
       </c>
     </row>
     <row r="1495" spans="1:12" x14ac:dyDescent="0.35">
@@ -59182,8 +59182,8 @@
       <c r="K1542">
         <v>0</v>
       </c>
-      <c r="L1542" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1542">
+        <v>0</v>
       </c>
     </row>
     <row r="1543" spans="1:12" x14ac:dyDescent="0.35">
@@ -67352,8 +67352,8 @@
       <c r="K1757">
         <v>0</v>
       </c>
-      <c r="L1757" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1757">
+        <v>0</v>
       </c>
     </row>
     <row r="1758" spans="1:12" x14ac:dyDescent="0.35">
@@ -68986,8 +68986,8 @@
       <c r="K1800">
         <v>0</v>
       </c>
-      <c r="L1800" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1800">
+        <v>0</v>
       </c>
     </row>
     <row r="1801" spans="1:12" x14ac:dyDescent="0.35">
@@ -69670,8 +69670,8 @@
       <c r="K1818">
         <v>0</v>
       </c>
-      <c r="L1818" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1818">
+        <v>0</v>
       </c>
     </row>
     <row r="1819" spans="1:12" x14ac:dyDescent="0.35">
@@ -71152,8 +71152,8 @@
       <c r="K1857">
         <v>0</v>
       </c>
-      <c r="L1857" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1857">
+        <v>0</v>
       </c>
     </row>
     <row r="1858" spans="1:12" x14ac:dyDescent="0.35">
@@ -75104,8 +75104,8 @@
       <c r="K1961">
         <v>0</v>
       </c>
-      <c r="L1961" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1961">
+        <v>0</v>
       </c>
     </row>
     <row r="1962" spans="1:12" x14ac:dyDescent="0.35">
@@ -75294,8 +75294,8 @@
       <c r="K1966">
         <v>0</v>
       </c>
-      <c r="L1966" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1966">
+        <v>0</v>
       </c>
     </row>
     <row r="1967" spans="1:12" x14ac:dyDescent="0.35">
@@ -76054,8 +76054,8 @@
       <c r="K1986">
         <v>0</v>
       </c>
-      <c r="L1986" t="e">
-        <v>#DIV/0!</v>
+      <c r="L1986">
+        <v>0</v>
       </c>
     </row>
     <row r="1987" spans="1:12" x14ac:dyDescent="0.35">
@@ -77612,8 +77612,8 @@
       <c r="K2027">
         <v>0</v>
       </c>
-      <c r="L2027" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2027">
+        <v>0</v>
       </c>
     </row>
     <row r="2028" spans="1:12" x14ac:dyDescent="0.35">
@@ -78828,8 +78828,8 @@
       <c r="K2059">
         <v>0</v>
       </c>
-      <c r="L2059" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2059">
+        <v>0</v>
       </c>
     </row>
     <row r="2060" spans="1:12" x14ac:dyDescent="0.35">
@@ -80842,8 +80842,8 @@
       <c r="K2112">
         <v>0</v>
       </c>
-      <c r="L2112" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2112">
+        <v>0</v>
       </c>
     </row>
     <row r="2113" spans="1:12" x14ac:dyDescent="0.35">
@@ -82172,8 +82172,8 @@
       <c r="K2147">
         <v>0</v>
       </c>
-      <c r="L2147" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2147">
+        <v>0</v>
       </c>
     </row>
     <row r="2148" spans="1:12" x14ac:dyDescent="0.35">
@@ -82286,8 +82286,8 @@
       <c r="K2150">
         <v>0</v>
       </c>
-      <c r="L2150" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2150">
+        <v>0</v>
       </c>
     </row>
     <row r="2151" spans="1:12" x14ac:dyDescent="0.35">
@@ -83616,8 +83616,8 @@
       <c r="K2185">
         <v>0</v>
       </c>
-      <c r="L2185" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2185">
+        <v>0</v>
       </c>
     </row>
     <row r="2186" spans="1:12" x14ac:dyDescent="0.35">
@@ -86428,8 +86428,8 @@
       <c r="K2259">
         <v>0</v>
       </c>
-      <c r="L2259" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2259">
+        <v>0</v>
       </c>
     </row>
     <row r="2260" spans="1:12" x14ac:dyDescent="0.35">
@@ -86618,8 +86618,8 @@
       <c r="K2264">
         <v>0</v>
       </c>
-      <c r="L2264" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2264">
+        <v>0</v>
       </c>
     </row>
     <row r="2265" spans="1:12" x14ac:dyDescent="0.35">
@@ -87036,8 +87036,8 @@
       <c r="K2275">
         <v>0</v>
       </c>
-      <c r="L2275" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2275">
+        <v>0</v>
       </c>
     </row>
     <row r="2276" spans="1:12" x14ac:dyDescent="0.35">
@@ -90228,8 +90228,8 @@
       <c r="K2359">
         <v>0</v>
       </c>
-      <c r="L2359" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2359">
+        <v>0</v>
       </c>
     </row>
     <row r="2360" spans="1:12" x14ac:dyDescent="0.35">
@@ -91026,8 +91026,8 @@
       <c r="K2380">
         <v>0</v>
       </c>
-      <c r="L2380" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2380">
+        <v>0</v>
       </c>
     </row>
     <row r="2381" spans="1:12" x14ac:dyDescent="0.35">
@@ -91064,8 +91064,8 @@
       <c r="K2381">
         <v>0</v>
       </c>
-      <c r="L2381" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2381">
+        <v>0</v>
       </c>
     </row>
     <row r="2382" spans="1:12" x14ac:dyDescent="0.35">
@@ -91710,8 +91710,8 @@
       <c r="K2398">
         <v>0</v>
       </c>
-      <c r="L2398" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2398">
+        <v>0</v>
       </c>
     </row>
     <row r="2399" spans="1:12" x14ac:dyDescent="0.35">
@@ -91824,8 +91824,8 @@
       <c r="K2401">
         <v>0</v>
       </c>
-      <c r="L2401" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2401">
+        <v>0</v>
       </c>
     </row>
     <row r="2402" spans="1:12" x14ac:dyDescent="0.35">
@@ -91900,8 +91900,8 @@
       <c r="K2403">
         <v>0</v>
       </c>
-      <c r="L2403" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2403">
+        <v>0</v>
       </c>
     </row>
     <row r="2404" spans="1:12" x14ac:dyDescent="0.35">
@@ -92052,8 +92052,8 @@
       <c r="K2407">
         <v>0</v>
       </c>
-      <c r="L2407" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2407">
+        <v>0</v>
       </c>
     </row>
     <row r="2408" spans="1:12" x14ac:dyDescent="0.35">
@@ -92888,8 +92888,8 @@
       <c r="K2429">
         <v>0</v>
       </c>
-      <c r="L2429" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2429">
+        <v>0</v>
       </c>
     </row>
     <row r="2430" spans="1:12" x14ac:dyDescent="0.35">
@@ -93458,8 +93458,8 @@
       <c r="K2444">
         <v>0</v>
       </c>
-      <c r="L2444" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2444">
+        <v>0</v>
       </c>
     </row>
     <row r="2445" spans="1:12" x14ac:dyDescent="0.35">
@@ -94066,8 +94066,8 @@
       <c r="K2460">
         <v>0</v>
       </c>
-      <c r="L2460" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2460">
+        <v>0</v>
       </c>
     </row>
     <row r="2461" spans="1:12" x14ac:dyDescent="0.35">
@@ -94294,8 +94294,8 @@
       <c r="K2466">
         <v>0</v>
       </c>
-      <c r="L2466" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2466">
+        <v>0</v>
       </c>
     </row>
     <row r="2467" spans="1:12" x14ac:dyDescent="0.35">
@@ -94522,8 +94522,8 @@
       <c r="K2472">
         <v>0</v>
       </c>
-      <c r="L2472" t="e">
-        <v>#DIV/0!</v>
+      <c r="L2472">
+        <v>0</v>
       </c>
     </row>
     <row r="2473" spans="1:12" x14ac:dyDescent="0.35">

</xml_diff>